<commit_message>
Train a Skill L3 Lower Body: 1 leg weighted horizontal back extension added (grade 2, coach standard)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yWLLpzw9R1iGhMPWXgZsW
</commit_message>
<xml_diff>
--- a/Train_A_Skill/Level3_Train_A_Skill_LowerBody.xlsx
+++ b/Train_A_Skill/Level3_Train_A_Skill_LowerBody.xlsx
@@ -1666,7 +1666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2390,17 +2390,17 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Deficit Deadlifts</t>
+          <t>1 leg weighted horizontal back extension</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>8 reps for 90% of bodyweight</t>
+          <t>10 reps for 5% bodyweight, avoid feet from turning out and hold extension at the top of the movement each rep</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>6–8 reps @ 35–90% BW</t>
+          <t>8–10 reps @ 2.5–5% BW</t>
         </is>
       </c>
     </row>
@@ -2412,17 +2412,17 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Deficit landmine SL deadlift</t>
+          <t>Deficit Deadlifts</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>8 reps each leg 50% of bodyweight</t>
+          <t>8 reps for 90% of bodyweight</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>6–8 reps each leg @ 20–50% BW</t>
+          <t>6–8 reps @ 35–90% BW</t>
         </is>
       </c>
     </row>
@@ -2434,17 +2434,17 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>1 leg deficit BB deadlift</t>
+          <t>Deficit landmine SL deadlift</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>8 reps each leg 45% of bodyweight</t>
+          <t>8 reps each leg 50% of bodyweight</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>6–8 reps each leg @ 20–45% BW</t>
+          <t>6–8 reps each leg @ 20–50% BW</t>
         </is>
       </c>
     </row>
@@ -2456,17 +2456,17 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Hands assisted full range nordic curl</t>
+          <t>1 leg deficit BB deadlift</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>10 reps</t>
+          <t>8 reps each leg 45% of bodyweight</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>6–10 reps</t>
+          <t>6–8 reps each leg @ 20–45% BW</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2478,17 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Assisted Razor Curls</t>
+          <t>Hands assisted full range nordic curl</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>12 reps</t>
+          <t>10 reps</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>6–12 reps</t>
+          <t>6–10 reps</t>
         </is>
       </c>
     </row>
@@ -2500,28 +2500,51 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
+          <t>Assisted Razor Curls</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>12 reps</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>6–12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>○  2</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
           <t>plantar flexion full range assisted nordic</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>10 reps</t>
         </is>
       </c>
-      <c r="D47" s="10" t="inlineStr">
+      <c r="D48" s="10" t="inlineStr">
         <is>
           <t>6–10 reps</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="8" customHeight="1"/>
+    <row r="49" ht="8" customHeight="1"/>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="46">
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="D27:F27"/>
     <mergeCell ref="D41:F41"/>
     <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D48:F48"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="D16:F16"/>
@@ -2598,6 +2621,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>